<commit_message>
Add remote access scripts
</commit_message>
<xml_diff>
--- a/программа.monthly-report.backup.xlsx
+++ b/программа.monthly-report.backup.xlsx
@@ -1735,7 +1735,6 @@
     <row r="14" ht="18" customHeight="1"/>
     <row r="15" ht="18" customHeight="1"/>
     <row r="16" ht="18" customHeight="1"/>
-    <row r="17"/>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
         <is>
@@ -1912,7 +1911,6 @@
     <row r="27" ht="18" customHeight="1"/>
     <row r="28" ht="18" customHeight="1"/>
     <row r="29" ht="18" customHeight="1"/>
-    <row r="30"/>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="21" t="inlineStr">
         <is>
@@ -2089,7 +2087,6 @@
     <row r="40" ht="18" customHeight="1"/>
     <row r="41" ht="18" customHeight="1"/>
     <row r="42" ht="18" customHeight="1"/>
-    <row r="43"/>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="21" t="inlineStr">
         <is>
@@ -2266,7 +2263,6 @@
     <row r="53" ht="18" customHeight="1"/>
     <row r="54" ht="18" customHeight="1"/>
     <row r="55" ht="18" customHeight="1"/>
-    <row r="56"/>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="21" t="inlineStr">
         <is>
@@ -2443,7 +2439,6 @@
     <row r="66" ht="18" customHeight="1"/>
     <row r="67" ht="18" customHeight="1"/>
     <row r="68" ht="18" customHeight="1"/>
-    <row r="69"/>
     <row r="70" ht="20" customHeight="1">
       <c r="A70" s="21" t="inlineStr">
         <is>
@@ -2745,28 +2740,6 @@
       </c>
       <c r="B81" t="n">
         <v>2</v>
-      </c>
-      <c r="C81" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="D81" t="n">
-        <v>11</v>
-      </c>
-      <c r="F81" t="n">
-        <v>25</v>
-      </c>
-      <c r="G81" t="n">
-        <v>9</v>
-      </c>
-      <c r="O81" t="inlineStr">
-        <is>
-          <t>25x9</t>
-        </is>
-      </c>
-      <c r="P81" t="inlineStr">
-        <is>
-          <t>Тест API</t>
-        </is>
       </c>
     </row>
     <row r="82">

</xml_diff>